<commit_message>
need to fix how attaching sensors to series comps
</commit_message>
<xml_diff>
--- a/Simulators/auxiliary_ship_data.xlsx
+++ b/Simulators/auxiliary_ship_data.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adware\Desktop\KISS\Simulators\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BB995FA-389B-4180-9026-FE539BBDB530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A162F086-D470-47AA-B724-6486F4D5F00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
+    <workbookView xWindow="0" yWindow="368" windowWidth="19200" windowHeight="11085" activeTab="3" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
   </bookViews>
   <sheets>
     <sheet name="machinery reliability data" sheetId="1" r:id="rId1"/>
     <sheet name="system structure data" sheetId="2" r:id="rId2"/>
     <sheet name="ship structure" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -542,15 +543,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F997A0B-9C86-4EC5-9A0F-10545207BFB0}">
   <dimension ref="A1:F37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" style="2" customWidth="1"/>
-    <col min="4" max="6" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.73046875" customWidth="1"/>
+    <col min="2" max="2" width="24.1328125" customWidth="1"/>
+    <col min="3" max="3" width="18.265625" style="2" customWidth="1"/>
+    <col min="4" max="6" width="18.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
@@ -570,7 +571,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
@@ -590,7 +591,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
@@ -610,7 +611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
@@ -630,7 +631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
@@ -650,7 +651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4</v>
       </c>
@@ -670,7 +671,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
@@ -690,7 +691,7 @@
         <v>0.997</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6</v>
       </c>
@@ -710,7 +711,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>7</v>
       </c>
@@ -730,7 +731,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>8</v>
       </c>
@@ -750,7 +751,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>9</v>
       </c>
@@ -770,7 +771,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>10</v>
       </c>
@@ -790,7 +791,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>11</v>
       </c>
@@ -810,7 +811,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>12</v>
       </c>
@@ -830,7 +831,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.45">
       <c r="C37" s="5"/>
     </row>
   </sheetData>
@@ -842,12 +843,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD4FF0A7-4C32-4212-8D10-DADC32F7B7B8}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="3" width="32.42578125" customWidth="1"/>
+    <col min="2" max="3" width="32.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -858,7 +859,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
@@ -869,7 +870,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
@@ -880,7 +881,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
@@ -891,7 +892,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
@@ -902,7 +903,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="D6" s="4"/>
     </row>
   </sheetData>
@@ -914,19 +915,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B338D18E-1C2C-4003-BC79-5462DE0704E2}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.1328125" customWidth="1"/>
+    <col min="2" max="2" width="30.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -934,4 +935,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A16644A-918D-4FF5-9CE2-44B4969116F9}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>